<commit_message>
ya guarda solo los datos escritos, pero no las formulas
</commit_message>
<xml_diff>
--- a/assets/contabilizacion.xlsx
+++ b/assets/contabilizacion.xlsx
@@ -989,8 +989,16 @@
       <c r="B2" s="36" t="n">
         <v>45236</v>
       </c>
-      <c r="C2" s="37" t="n"/>
-      <c r="D2" s="37" t="n"/>
+      <c r="C2" s="37" t="inlineStr">
+        <is>
+          <t>nnnn</t>
+        </is>
+      </c>
+      <c r="D2" s="37" t="inlineStr">
+        <is>
+          <t>21244</t>
+        </is>
+      </c>
       <c r="E2" s="28" t="inlineStr">
         <is>
           <t>adelanto jose</t>
@@ -1028,8 +1036,16 @@
       <c r="B3" s="36" t="n">
         <v>45236</v>
       </c>
-      <c r="C3" s="37" t="n"/>
-      <c r="D3" s="37" t="n"/>
+      <c r="C3" s="37" t="inlineStr">
+        <is>
+          <t>asfg</t>
+        </is>
+      </c>
+      <c r="D3" s="37" t="inlineStr">
+        <is>
+          <t>fnn</t>
+        </is>
+      </c>
       <c r="E3" s="28" t="inlineStr">
         <is>
           <t>aveo correa reparitcion 300 nequi 40 efecitvo</t>
@@ -1069,7 +1085,11 @@
       <c r="B4" s="36" t="n">
         <v>45236</v>
       </c>
-      <c r="C4" s="37" t="n"/>
+      <c r="C4" s="37" t="inlineStr">
+        <is>
+          <t>sdg</t>
+        </is>
+      </c>
       <c r="D4" s="37" t="n"/>
       <c r="E4" s="28" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
usar container para que se expanda a todo el espacio y usar python 3.11
</commit_message>
<xml_diff>
--- a/assets/contabilizacion.xlsx
+++ b/assets/contabilizacion.xlsx
@@ -985,7 +985,11 @@
       </c>
     </row>
     <row r="2" ht="19.5" customHeight="1">
-      <c r="A2" s="36" t="n"/>
+      <c r="A2" s="36" t="inlineStr">
+        <is>
+          <t>hola</t>
+        </is>
+      </c>
       <c r="B2" s="36" t="n">
         <v>45236</v>
       </c>

</xml_diff>

<commit_message>
poner de nuevo a que e = sirva
</commit_message>
<xml_diff>
--- a/assets/contabilizacion.xlsx
+++ b/assets/contabilizacion.xlsx
@@ -1130,7 +1130,11 @@
       <c r="B5" s="36" t="n">
         <v>45236</v>
       </c>
-      <c r="C5" s="37" t="n"/>
+      <c r="C5" s="37" t="inlineStr">
+        <is>
+          <t>dasdgd</t>
+        </is>
+      </c>
       <c r="D5" s="37" t="inlineStr">
         <is>
           <t>shdjfh</t>
@@ -1257,7 +1261,9 @@
       <c r="B8" s="36" t="n">
         <v>45236</v>
       </c>
-      <c r="C8" s="37" t="n"/>
+      <c r="C8" s="37" t="n">
+        <v>21333</v>
+      </c>
       <c r="D8" s="37" t="n"/>
       <c r="E8" s="28" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
ahora guarda formulas en su cell.formula
</commit_message>
<xml_diff>
--- a/assets/contabilizacion.xlsx
+++ b/assets/contabilizacion.xlsx
@@ -993,7 +993,10 @@
           <t>2023-11-06 00:00:00</t>
         </is>
       </c>
-      <c r="C2" s="37" t="n"/>
+      <c r="C2" s="37">
+        <f>2345*45643</f>
+        <v/>
+      </c>
       <c r="D2" s="37" t="inlineStr">
         <is>
           <t>21244</t>
@@ -1038,15 +1041,13 @@
       <c r="B3" s="36" t="n">
         <v>45236</v>
       </c>
-      <c r="C3" s="37" t="inlineStr">
-        <is>
-          <t>65</t>
-        </is>
-      </c>
-      <c r="D3" s="37" t="inlineStr">
-        <is>
-          <t>fnn</t>
-        </is>
+      <c r="C3" s="37">
+        <f>C2*D2</f>
+        <v/>
+      </c>
+      <c r="D3" s="37">
+        <f>C2+C7</f>
+        <v/>
       </c>
       <c r="E3" s="28" t="inlineStr">
         <is>
@@ -1087,12 +1088,15 @@
       <c r="B4" s="36" t="n">
         <v>45236</v>
       </c>
-      <c r="C4" s="37" t="inlineStr">
-        <is>
-          <t>sdg</t>
-        </is>
-      </c>
-      <c r="D4" s="37" t="n"/>
+      <c r="C4" s="37">
+        <f>23453*336543</f>
+        <v/>
+      </c>
+      <c r="D4" s="37" t="inlineStr">
+        <is>
+          <t>a</t>
+        </is>
+      </c>
       <c r="E4" s="28" t="inlineStr">
         <is>
           <t>aveo correa reparitcion 300 nequi 40 efecitvo</t>
@@ -1222,7 +1226,9 @@
       <c r="B7" s="36" t="n">
         <v>45236</v>
       </c>
-      <c r="C7" s="37" t="n"/>
+      <c r="C7" s="37" t="n">
+        <v>75816</v>
+      </c>
       <c r="D7" s="37" t="n"/>
       <c r="E7" s="28" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
ahora guarda bien los datos y almacena sus valores y sus formulas en cell.content.value y  cell.formula!!!
</commit_message>
<xml_diff>
--- a/assets/contabilizacion.xlsx
+++ b/assets/contabilizacion.xlsx
@@ -993,9 +993,10 @@
           <t>2023-11-06 00:00:00</t>
         </is>
       </c>
-      <c r="C2" s="37">
-        <f>2345*45643</f>
-        <v/>
+      <c r="C2" s="37" t="inlineStr">
+        <is>
+          <t>veapues</t>
+        </is>
       </c>
       <c r="D2" s="37" t="inlineStr">
         <is>
@@ -1041,12 +1042,13 @@
       <c r="B3" s="36" t="n">
         <v>45236</v>
       </c>
-      <c r="C3" s="37">
-        <f>C2*D2</f>
-        <v/>
+      <c r="C3" s="37" t="inlineStr">
+        <is>
+          <t>5hyd</t>
+        </is>
       </c>
       <c r="D3" s="37">
-        <f>C2+C7</f>
+        <f>2345*34421-2314</f>
         <v/>
       </c>
       <c r="E3" s="28" t="inlineStr">
@@ -1141,7 +1143,7 @@
       </c>
       <c r="D5" s="37" t="inlineStr">
         <is>
-          <t>shdjfh</t>
+          <t>assd</t>
         </is>
       </c>
       <c r="E5" s="28" t="inlineStr">
@@ -1653,9 +1655,14 @@
           <t xml:space="preserve">tubo paso agua corsa^ </t>
         </is>
       </c>
-      <c r="C2" s="28" t="n"/>
-      <c r="D2" s="16" t="n">
-        <v>35000</v>
+      <c r="C2" s="28" t="inlineStr">
+        <is>
+          <t>mirandacon</t>
+        </is>
+      </c>
+      <c r="D2" s="16">
+        <f>2355*2345</f>
+        <v/>
       </c>
       <c r="E2" s="16" t="n">
         <v>9800</v>
@@ -1697,8 +1704,9 @@
           <t>PARTMO</t>
         </is>
       </c>
-      <c r="D3" s="16" t="n">
-        <v>15000</v>
+      <c r="D3" s="16">
+        <f>E2*E4</f>
+        <v/>
       </c>
       <c r="E3" s="16" t="n">
         <v>10600</v>
@@ -3855,13 +3863,14 @@
       <c r="B2" s="18" t="n">
         <v>166</v>
       </c>
-      <c r="C2" s="15" t="inlineStr">
-        <is>
-          <t>323</t>
-        </is>
-      </c>
-      <c r="D2" s="13" t="n">
-        <v>0</v>
+      <c r="C2" s="15">
+        <f>B2*I3</f>
+        <v/>
+      </c>
+      <c r="D2" s="13" t="inlineStr">
+        <is>
+          <t>miraculous</t>
+        </is>
       </c>
       <c r="E2" s="15" t="inlineStr">
         <is>
@@ -3914,10 +3923,9 @@
           <t>varilla medidora de aceite megane clio symbol</t>
         </is>
       </c>
-      <c r="D3" s="14" t="inlineStr">
-        <is>
-          <t>CYT</t>
-        </is>
+      <c r="D3" s="14">
+        <f>I3*I4</f>
+        <v/>
       </c>
       <c r="E3" s="15" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
ahora aparece cuadro guia de la formula o value arriba
</commit_message>
<xml_diff>
--- a/assets/contabilizacion.xlsx
+++ b/assets/contabilizacion.xlsx
@@ -1012,7 +1012,10 @@
       <c r="G2" s="38" t="n">
         <v>-30000</v>
       </c>
-      <c r="H2" s="16" t="n"/>
+      <c r="H2" s="16">
+        <f>456*3456</f>
+        <v/>
+      </c>
       <c r="I2" s="16" t="n"/>
       <c r="J2" s="39" t="n"/>
       <c r="K2" s="40" t="n"/>

</xml_diff>

<commit_message>
ahora es mas rapido al solo guardar lo modificado y no guardar todo completo como tal
</commit_message>
<xml_diff>
--- a/assets/contabilizacion.xlsx
+++ b/assets/contabilizacion.xlsx
@@ -1111,7 +1111,11 @@
         <v>40000</v>
       </c>
       <c r="G4" s="38" t="n"/>
-      <c r="H4" s="16" t="n"/>
+      <c r="H4" s="16" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="I4" s="16" t="n"/>
       <c r="J4" s="39" t="n"/>
       <c r="K4" s="40" t="n"/>
@@ -1158,7 +1162,10 @@
         <v>100000</v>
       </c>
       <c r="G5" s="38" t="n"/>
-      <c r="H5" s="16" t="n"/>
+      <c r="H5" s="16">
+        <f>2356*4432</f>
+        <v/>
+      </c>
       <c r="I5" s="16" t="n"/>
       <c r="J5" s="39" t="n"/>
       <c r="K5" s="40" t="n"/>
@@ -1203,7 +1210,10 @@
       <c r="G6" s="38" t="n">
         <v>-15000</v>
       </c>
-      <c r="H6" s="16" t="n"/>
+      <c r="H6" s="16">
+        <f>G6+3443021</f>
+        <v/>
+      </c>
       <c r="I6" s="16" t="n"/>
       <c r="J6" s="39" t="n"/>
       <c r="K6" s="40" t="n"/>

</xml_diff>

<commit_message>
colocar logs en ios
</commit_message>
<xml_diff>
--- a/assets/contabilizacion.xlsx
+++ b/assets/contabilizacion.xlsx
@@ -1254,7 +1254,11 @@
       <c r="G7" s="38" t="n">
         <v>-38000</v>
       </c>
-      <c r="H7" s="16" t="n"/>
+      <c r="H7" s="16" t="inlineStr">
+        <is>
+          <t>h</t>
+        </is>
+      </c>
       <c r="I7" s="16" t="n"/>
       <c r="J7" s="39" t="n"/>
       <c r="K7" s="40" t="n"/>
@@ -1775,7 +1779,10 @@
           <t>8D-7</t>
         </is>
       </c>
-      <c r="H4" s="28" t="n"/>
+      <c r="H4" s="28">
+        <f>E2*L4+D6-A4*6</f>
+        <v/>
+      </c>
       <c r="I4" s="29" t="n"/>
       <c r="J4" s="28" t="n"/>
       <c r="K4" s="16" t="n"/>

</xml_diff>

<commit_message>
cambiar forma del yml
</commit_message>
<xml_diff>
--- a/assets/contabilizacion.xlsx
+++ b/assets/contabilizacion.xlsx
@@ -1200,7 +1200,10 @@
           <t>wueye</t>
         </is>
       </c>
-      <c r="D6" s="37" t="n"/>
+      <c r="D6" s="37">
+        <f>C4*45</f>
+        <v/>
+      </c>
       <c r="E6" s="28" t="inlineStr">
         <is>
           <t>adelanto edison</t>

</xml_diff>

<commit_message>
cambia el estilo de las fechas
</commit_message>
<xml_diff>
--- a/assets/contabilizacion.xlsx
+++ b/assets/contabilizacion.xlsx
@@ -1089,7 +1089,11 @@
       <c r="AC3" s="38" t="n"/>
     </row>
     <row r="4" ht="19.5" customHeight="1">
-      <c r="A4" s="36" t="n"/>
+      <c r="A4" s="36" t="inlineStr">
+        <is>
+          <t>15-June-2001</t>
+        </is>
+      </c>
       <c r="B4" s="36" t="n">
         <v>45236</v>
       </c>

</xml_diff>

<commit_message>
probar evaluar otra opcion
</commit_message>
<xml_diff>
--- a/assets/contabilizacion.xlsx
+++ b/assets/contabilizacion.xlsx
@@ -639,6 +639,10 @@
       <c r="E4" s="5" t="n">
         <v>300000</v>
       </c>
+      <c r="F4">
+        <f>23*432</f>
+        <v/>
+      </c>
       <c r="G4" s="5">
         <f>SUM(E4:F4)</f>
         <v/>
@@ -685,6 +689,10 @@
         <is>
           <t>gastos representacion</t>
         </is>
+      </c>
+      <c r="E6">
+        <f>E5+E2</f>
+        <v/>
       </c>
       <c r="F6" s="5" t="n">
         <v>-1000</v>

</xml_diff>

<commit_message>
separar con re match mejor las formulas
</commit_message>
<xml_diff>
--- a/assets/contabilizacion.xlsx
+++ b/assets/contabilizacion.xlsx
@@ -672,6 +672,10 @@
         <f>SUM(E5:F5)</f>
         <v/>
       </c>
+      <c r="I5">
+        <f>80SUM/8E4:F49</f>
+        <v/>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="n">

</xml_diff>

<commit_message>
ahora sirve bien la sum
</commit_message>
<xml_diff>
--- a/assets/contabilizacion.xlsx
+++ b/assets/contabilizacion.xlsx
@@ -1381,6 +1381,10 @@
           <t>9c-8</t>
         </is>
       </c>
+      <c r="H6">
+        <f>SUM(D2:E12)</f>
+        <v/>
+      </c>
       <c r="I6">
         <f>SUMIFS('entradas y salidas'!I:I,'entradas y salidas'!B:B,productos!A6)</f>
         <v/>

</xml_diff>

<commit_message>
este sumifs tiene una funcion de momento
</commit_message>
<xml_diff>
--- a/assets/contabilizacion.xlsx
+++ b/assets/contabilizacion.xlsx
@@ -705,6 +705,11 @@
         <f>SUM(E6:F6)</f>
         <v/>
       </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>0SUM8E2:F209</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="n">
@@ -728,6 +733,10 @@
       </c>
       <c r="G7" s="5">
         <f>SUM(E7:F7)</f>
+        <v/>
+      </c>
+      <c r="I7">
+        <f>SUM(E2:F9)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
manejar con mayor facilidad las referencias
</commit_message>
<xml_diff>
--- a/assets/contabilizacion.xlsx
+++ b/assets/contabilizacion.xlsx
@@ -705,10 +705,9 @@
         <f>SUM(E6:F6)</f>
         <v/>
       </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>0SUM8E2:F209</t>
-        </is>
+      <c r="I6">
+        <f>TEXT(A2;"dddd")</f>
+        <v/>
       </c>
     </row>
     <row r="7">

</xml_diff>